<commit_message>
Programı yeni zaman kurallarına göre güncelle: ödev+tekrar 1.5 saat, ek çalışma 2 saat, 22:00 uyku
Tüm hafta için sabit bir saat şablonu kuruldu: 17:30 okul çıkışı,
17:40-18:25 günlük ödev, üç adet ek çalışma bloğu (toplam 2 saat),
21:10-21:55 günlük tekrar, 21:55-22:00 yatış hazırlığı ve 22:00 uyku.
Haftalık ders dağılımı özeti ve güncellenmiş kullanım rehberi eklendi.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7UkXbn3U8T5AXkNxv5cKV
</commit_message>
<xml_diff>
--- a/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
+++ b/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Nasıl Düzenlenir" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,49 +56,65 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3B57"/>
-      <sz val="9"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0037474F"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A237E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00BF360C"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="000D47A1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00BF360C"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001B5E20"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="004A148C"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0037474F"/>
-      <sz val="9"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00827717"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00004D40"/>
-      <sz val="9"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00311B92"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -114,6 +130,29 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3B57"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0037474F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A237E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00455A64"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00BF360C"/>
       <sz val="10"/>
     </font>
@@ -135,12 +174,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00455A64"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00827717"/>
       <sz val="10"/>
     </font>
@@ -148,6 +181,18 @@
       <name val="Arial"/>
       <color rgb="0000695C"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00311B92"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00546E7A"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -175,7 +220,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -214,8 +259,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BBDEFB"/>
-        <bgColor rgb="00BBDEFB"/>
+        <fgColor rgb="00CFD8DC"/>
+        <bgColor rgb="00CFD8DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B3C7E6"/>
+        <bgColor rgb="00B3C7E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -226,6 +277,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C8E6C9"/>
         <bgColor rgb="00C8E6C9"/>
       </patternFill>
@@ -256,8 +313,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00CFCFEA"/>
+        <bgColor rgb="00CFCFEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3B57"/>
         <bgColor rgb="001F3B57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
+        <bgColor rgb="00F5F7FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -287,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -326,51 +395,80 @@
     <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -739,10 +837,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -777,7 +875,7 @@
       <c r="A2" s="4" t="n"/>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Rehber Öğretmen: Merve Çelik</t>
+          <t>Rehber Öğretmen: Merve Çelik   |   Program: 17:30 Okul Çıkışı – 22:00 Uyku</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -805,553 +903,745 @@
       <c r="G3" s="8" t="n"/>
       <c r="H3" s="8" t="n"/>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Renk Kodları:</t>
+          <t>Renk
+Kodları:</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
+          <t>Giriş / Dinlenme</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Günlük Ödev</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Matematik</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
           <t>Türkçe</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>Matematik</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Fen Bilimleri</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Sosyal Bilgiler</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Mola</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>Yemek / Serbest</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>Tekrar / Değerlendirme</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="17" t="inlineStr"/>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Yemek</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Günlük Tekrar</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Yatış Hazırlığı</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr"/>
+      <c r="F5" s="21" t="inlineStr"/>
+      <c r="G5" s="21" t="inlineStr"/>
+      <c r="H5" s="21" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Zaman Bloğu</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Pazartesi</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>Salı</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Çarşamba</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>Perşembe</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F6" s="23" t="inlineStr">
         <is>
           <t>Cuma</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>Cumartesi</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>Pazar</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Blok 1
-(Ders Çalışması)</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>18:30–19:10
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Giriş / Dinlenme</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>17:30–17:40
+Eve Varış /
+Dinlenme</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Günlük Ödev</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>17:40–18:25
+Günlük Ödevler</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="inlineStr">
+        <is>
+          <t>18:25–18:35
+Mola</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 1</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>18:35–19:20
 Matematik
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>18:30–19:10
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>18:35–19:20
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>18:30–19:10
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>18:35–19:20
+Matematik
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>18:35–19:20
+Sosyal Bilgiler
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>18:35–19:20
+Fen Bilimleri
+Test Çözümü</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>18:35–19:20
+Matematik
+Yanlış Analizi</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>18:35–19:20
+Matematik
+Genel Tekrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Yemek</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>19:20–19:45
+Yemek</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 2</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>19:45–20:30
+Türkçe
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>19:45–20:30
+Matematik
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>19:45–20:30
+Fen Bilimleri
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>19:45–20:30
 Matematik
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>18:30–19:10
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>19:45–20:30
+Türkçe
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>19:45–20:30
 Sosyal Bilgiler
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>18:30–19:10
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>19:45–20:30
+Türkçe
+Genel Tekrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>20:30–20:40
+Mola</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 3</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Fen Bilimleri
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>10:00–10:40
-Matematik
-Yanlış Analizi</t>
-        </is>
-      </c>
-      <c r="H6" s="19" t="inlineStr">
-        <is>
-          <t>10:00–10:40
-Matematik
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Mola</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>19:10–19:20
-Mola</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>19:10–19:20
-Mola</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>19:10–19:20
-Mola</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>19:10–19:20
-Mola</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>19:10–19:20
-Mola</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>10:40–10:50
-Mola</t>
-        </is>
-      </c>
-      <c r="H7" s="23" t="inlineStr">
-        <is>
-          <t>10:40–10:50
-Mola</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Blok 2
-(Ders Çalışması)</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>19:20–20:00
-Türkçe
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>19:20–20:00
-Matematik
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="D8" s="22" t="inlineStr">
-        <is>
-          <t>19:20–20:00
-Fen Bilimleri
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>19:20–20:00
-Matematik
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>20:40–21:10
+Sosyal Bilgiler
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Türkçe
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
-        <is>
-          <t>10:50–11:30
-Sosyal Bilgiler
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>10:50–11:30
-Türkçe
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Yemek /
-Uzun Mola</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>20:00–20:30
-Yemek / Uzun Mola</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>20:00–20:30
-Yemek / Uzun Mola</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>20:00–20:30
-Yemek / Uzun Mola</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>20:00–20:30
-Yemek / Uzun Mola</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>20:00–20:30
-Yemek / Uzun Mola</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>11:30–15:00
-Serbest Zaman /
-Aile / Hobi</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="inlineStr">
-        <is>
-          <t>11:30–15:00
-Serbest Zaman /
-Aile</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Blok 3
-(Ders Çalışması)</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>20:30–21:10
-Fen Bilimleri
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>20:30–21:10
-Sosyal Bilgiler
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>20:30–21:10
-Türkçe
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>20:30–21:10
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>20:30–21:10
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Matematik
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G10" s="22" t="inlineStr">
-        <is>
-          <t>15:00–15:40
+      <c r="G14" s="31" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Fen Bilimleri
 Test Çözümü</t>
         </is>
       </c>
-      <c r="H10" s="22" t="inlineStr">
-        <is>
-          <t>15:00–15:40
+      <c r="H14" s="31" t="inlineStr">
+        <is>
+          <t>20:40–21:10
 Fen Bil. &amp; Sosyal Bil.
 Genel Tekrar</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Mola</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>21:10–21:20
-Mola</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>21:10–21:20
-Mola</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>21:10–21:20
-Mola</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>21:10–21:20
-Mola</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>21:10–21:20
-Mola</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>15:40–15:50
-Mola</t>
-        </is>
-      </c>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>15:40–15:50
-Mola</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Kısa Tekrar /
-Değerlendirme</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr">
-        <is>
-          <t>21:20–21:45
-Türkçe
-Kısa Tekrar (Kelime-Deyim)</t>
-        </is>
-      </c>
-      <c r="C12" s="25" t="inlineStr">
-        <is>
-          <t>21:20–21:45
-Serbest Okuma
-(Kitap)</t>
-        </is>
-      </c>
-      <c r="D12" s="25" t="inlineStr">
-        <is>
-          <t>21:20–21:45
-Matematik
-Yanlış Analizi</t>
-        </is>
-      </c>
-      <c r="E12" s="25" t="inlineStr">
-        <is>
-          <t>21:20–21:45
-Fen Bilimleri
-Kısa Tekrar</t>
-        </is>
-      </c>
-      <c r="F12" s="25" t="inlineStr">
-        <is>
-          <t>21:20–21:45
-Haftalık Genel
-Değerlendirme</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>15:50–16:30
-Türkçe
-Test Çözümü</t>
-        </is>
-      </c>
-      <c r="H12" s="25" t="inlineStr">
-        <is>
-          <t>15:50–16:30
-Haftalık Planlama /
-Değerlendirme</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="26" t="inlineStr">
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Günlük Tekrar</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>21:10–21:55
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Yatış Hazırlığı</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>21:55–22:00
+Yatış Hazırlığı
+→ 22:00 Uyku</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>Haftalık Ek Çalışma Dağılımı  —  Matematik: 7  |  Türkçe: 6  |  Fen Bilimleri: 5  |  Sosyal Bilgiler: 3   (Günlük Ödev + Günlük Tekrar: 1.5 saat, Ek Çalışma: 2 saat/gün)</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="n"/>
+      <c r="C18" s="36" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="36" t="n"/>
+      <c r="F18" s="36" t="n"/>
+      <c r="G18" s="36" t="n"/>
+      <c r="H18" s="36" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>NOTLAR</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
-      <c r="H14" s="27" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="28" t="inlineStr"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="28" t="inlineStr"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="28" t="inlineStr"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="B20" s="38" t="n"/>
+      <c r="C20" s="38" t="n"/>
+      <c r="D20" s="38" t="n"/>
+      <c r="E20" s="38" t="n"/>
+      <c r="F20" s="38" t="n"/>
+      <c r="G20" s="38" t="n"/>
+      <c r="H20" s="38" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="39" t="inlineStr"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="39" t="inlineStr"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="39" t="inlineStr"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="40" t="inlineStr">
         <is>
           <t>“Düzenli çalışma, küçük adımların büyük sonuçlara dönüşmesidir.”</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="A26" s="41" t="inlineStr">
         <is>
           <t>TED Okulları  |  Rehberlik Servisi  |  Hazırlayan: Merve Çelik</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
-      <c r="H20" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
+      <c r="H26" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -1364,128 +1654,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="31" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Programı Nasıl Düzenlersiniz?</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="43" t="inlineStr">
+        <is>
+          <t>• Zaman Yapısı</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>Program 17:30 okul çıkışından 22:00 uyku saatine kadar sabit bir çerçeve üzerine kuruludur: Günlük Ödev + Günlük Tekrar toplam 1.5 saat, Ek Çalışma (3 blok) toplam 2 saat. İhtiyaca göre 2-3 saat aralığında uzatılabilir; bunun için Ek Çalışma bloklarının süresini ve Mola/Yemek sürelerini kısaltıp uzatarak yeniden dengeleyebilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>• Ders Saatleri</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>Her hücredeki saat aralığını (örn. 18:30–19:10) doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
-        <is>
-          <t>• Dersler ve Konular</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>"Haftalık Program" sayfasındaki her hücreye dersin adını ve yapılacak çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>Her hücredeki saat aralığını (örn. 18:35–19:20) doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="32" t="inlineStr">
-        <is>
-          <t>• Çalışma Süreleri</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>Blok başlıkları (Blok 1, Blok 2, Blok 3) ve mola süreleri satırlardaki saatleri değiştirerek yeniden ayarlanabilir.</t>
+      <c r="A9" s="43" t="inlineStr">
+        <is>
+          <t>• Ek Çalışma İçeriği</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>"Ek Çalışma 1/2/3" satırlarındaki hücrelere dersin adını ve çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="32" t="inlineStr">
-        <is>
-          <t>• Öğrenciye Özel Görevler</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>"Kısa Tekrar / Değerlendirme" satırı ve NOTLAR bölümü, öğrenciye özel ek görev veya hatırlatma yazmak için kullanılabilir.</t>
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>• Uyku Saati</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>Program 22:00'de uyku hedefiyle tasarlanmıştır. Yatış saatini değiştirmek isterseniz son satırdaki "Yatış Hazırlığı" bloğunun saatini güncelleyip diğer blokları buna göre kaydırın.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>• Hafta İçi / Hafta Sonu</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>Cumartesi ve Pazar sütunlarındaki saatler, hafta içine göre daha esnek planlanmıştır; ihtiyaca göre yeniden düzenlenebilir.</t>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>Program şu an tüm hafta için aynı saat şablonunu kullanır (tutarlı uyku düzeni için). Hafta sonu daha esnek olmasını isterseniz Cumartesi/Pazar sütunlarındaki saatleri ayrı ayrı değiştirebilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>• Renk Kodları</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>Her ders türü farklı bir renkle gösterilir (bkz. sayfa üstündeki 'Renk Kodları' satırı). Yeni bir hücre eklerken ilgili dersin rengini Hücre &gt; Dolgu Rengi seçeneğinden uygulayabilirsiniz.</t>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>Her blok türü farklı bir renkle gösterilir (bkz. sayfa üstündeki 'Renk Kodları' satırları).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="43" t="inlineStr">
         <is>
           <t>• Logo Alanı</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Sol üst köşedeki gri kutu TED okul logosu için ayrılmıştır. Logo görseli temin edildiğinde Ekle &gt; Resim ile bu alana yerleştirilebilir; kutu daha sonra silinebilir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="32" t="inlineStr">
-        <is>
-          <t>• Öğrenci / Hafta Bilgisi</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>Başlık altındaki 'Öğrenci Adı Soyadı' ve 'Hafta / Tarih Aralığı' alanları her hafta güncellenebilir.</t>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>Sol üst köşedeki gri kutu TED okul logosu için ayrılmıştır. Logo görseli temin edildiğinde Ekle &gt; Resim ile bu alana yerleştirilebilir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eve dönüşte 1 saat dinlenme ekle, ek çalışmayı 1.5 saate dengele
17:30-22:00 penceresi artık şöyle bölünüyor: 1 saat dinlenme,
1.5 saat günlük ödev+tekrar (45+45 dk), 1.5 saat ek çalışma
(2x45 dk), kısa molalar, 15 dk yemek ve yatış hazırlığı — toplam
tam 270 dakika, 22:00 uyku hedefini koruyor.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7UkXbn3U8T5AXkNxv5cKV
</commit_message>
<xml_diff>
--- a/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
+++ b/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Nasıl Düzenlenir" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -163,11 +163,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="004A148C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="001B5E20"/>
       <sz val="10"/>
     </font>
@@ -175,6 +170,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00827717"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="004A148C"/>
       <sz val="10"/>
     </font>
     <font>
@@ -435,13 +435,13 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -875,7 +875,7 @@
       <c r="A2" s="4" t="n"/>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Rehber Öğretmen: Merve Çelik   |   Program: 17:30 Okul Çıkışı – 22:00 Uyku</t>
+          <t>Rehber Öğretmen: Merve Çelik   |   17:30 Okul Çıkışı → 1 sa Dinlenme → 22:00 Uyku</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Giriş / Dinlenme</t>
@@ -1018,55 +1018,55 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
+Dinlenme (1 sa)</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>17:30–17:40
+          <t>17:30–18:30
 Eve Varış /
-Dinlenme</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
+Dinlenme (1 sa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Günlük Ödev</t>
@@ -1074,48 +1074,48 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>17:40–18:25
+          <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Mola</t>
@@ -1123,44 +1123,44 @@
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
       <c r="H9" s="27" t="inlineStr">
         <is>
-          <t>18:25–18:35
-Mola</t>
+          <t>19:15–19:20
+Kısa Mola</t>
         </is>
       </c>
     </row>
@@ -1172,313 +1172,257 @@
       </c>
       <c r="B10" s="28" t="inlineStr">
         <is>
-          <t>18:35–19:20
+          <t>19:20–20:05
 Matematik
 Konu Tekrarı</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>18:35–19:20
+          <t>19:20–20:05
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>18:35–19:20
+          <t>19:20–20:05
 Matematik
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr">
-        <is>
-          <t>18:35–19:20
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>19:20–20:05
+Türkçe
+Konu Tekrarı</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>19:20–20:05
+Fen Bilimleri
+Test Çözümü</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>19:20–20:05
+Matematik
+Yanlış Analizi</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>19:20–20:05
+Matematik
+Genel Tekrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Yemek</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>20:05–20:20
+Yemek</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 2</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>20:20–21:05
+Türkçe
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>20:20–21:05
+Matematik
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>20:20–21:05
+Fen Bilimleri
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>20:20–21:05
 Sosyal Bilgiler
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="F10" s="31" t="inlineStr">
-        <is>
-          <t>18:35–19:20
-Fen Bilimleri
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>20:20–21:05
+Türkçe
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t>18:35–19:20
-Matematik
-Yanlış Analizi</t>
-        </is>
-      </c>
-      <c r="H10" s="28" t="inlineStr">
-        <is>
-          <t>18:35–19:20
-Matematik
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>Yemek</t>
-        </is>
-      </c>
-      <c r="B11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="C11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="D11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="E11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="F11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="G11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-      <c r="H11" s="32" t="inlineStr">
-        <is>
-          <t>19:20–19:45
-Yemek</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>Ek Çalışma 2</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Türkçe
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Matematik
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Fen Bilimleri
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Matematik
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Türkçe
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="G12" s="30" t="inlineStr">
-        <is>
-          <t>19:45–20:30
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>20:20–21:05
 Sosyal Bilgiler
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="H12" s="29" t="inlineStr">
-        <is>
-          <t>19:45–20:30
-Türkçe
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>Mola</t>
-        </is>
-      </c>
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="C13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="D13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="E13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="G13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="inlineStr">
-        <is>
-          <t>20:30–20:40
-Mola</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Ek Çalışma 3</t>
-        </is>
-      </c>
-      <c r="B14" s="31" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Fen Bilimleri
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Sosyal Bilgiler
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="D14" s="29" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Türkçe
-Test Çözümü</t>
-        </is>
-      </c>
-      <c r="E14" s="29" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Türkçe
-Konu Tekrarı</t>
-        </is>
-      </c>
-      <c r="F14" s="28" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Matematik
-Test Çözümü</t>
-        </is>
-      </c>
-      <c r="G14" s="31" t="inlineStr">
-        <is>
-          <t>20:40–21:10
-Fen Bilimleri
-Test Çözümü</t>
-        </is>
-      </c>
-      <c r="H14" s="31" t="inlineStr">
-        <is>
-          <t>20:40–21:10
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>20:20–21:05
 Fen Bil. &amp; Sosyal Bil.
 Genel Tekrar</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>21:05–21:10
+Kısa Mola</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Günlük Tekrar</t>
         </is>
       </c>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="D15" s="33" t="inlineStr">
+      <c r="D14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="E15" s="33" t="inlineStr">
+      <c r="E14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="F15" s="33" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="G15" s="33" t="inlineStr">
+      <c r="G14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="H15" s="33" t="inlineStr">
+      <c r="H14" s="33" t="inlineStr">
         <is>
           <t>21:10–21:55
 Günlük Tekrar
@@ -1486,55 +1430,55 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="A16" s="24" t="inlineStr">
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Yatış Hazırlığı</t>
         </is>
       </c>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr">
+      <c r="D15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="E16" s="34" t="inlineStr">
+      <c r="E15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="F16" s="34" t="inlineStr">
+      <c r="F15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="G16" s="34" t="inlineStr">
+      <c r="G15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="H16" s="34" t="inlineStr">
+      <c r="H15" s="34" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
@@ -1542,33 +1486,43 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="35" t="inlineStr">
-        <is>
-          <t>Haftalık Ek Çalışma Dağılımı  —  Matematik: 7  |  Türkçe: 6  |  Fen Bilimleri: 5  |  Sosyal Bilgiler: 3   (Günlük Ödev + Günlük Tekrar: 1.5 saat, Ek Çalışma: 2 saat/gün)</t>
-        </is>
-      </c>
-      <c r="B18" s="36" t="n"/>
-      <c r="C18" s="36" t="n"/>
-      <c r="D18" s="36" t="n"/>
-      <c r="E18" s="36" t="n"/>
-      <c r="F18" s="36" t="n"/>
-      <c r="G18" s="36" t="n"/>
-      <c r="H18" s="36" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="37" t="inlineStr">
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>Haftalık Ek Çalışma Dağılımı  —  Matematik: 5  |  Türkçe: 4  |  Fen Bilimleri: 3  |  Sosyal Bilgiler: 2   (Dinlenme: 1 saat, Günlük Ödev + Günlük Tekrar: 1.5 saat, Ek Çalışma: 1.5 saat/gün, Uyku: 22:00)</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="n"/>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
+      <c r="G17" s="36" t="n"/>
+      <c r="H17" s="36" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>NOTLAR</t>
         </is>
       </c>
-      <c r="B20" s="38" t="n"/>
-      <c r="C20" s="38" t="n"/>
-      <c r="D20" s="38" t="n"/>
-      <c r="E20" s="38" t="n"/>
-      <c r="F20" s="38" t="n"/>
-      <c r="G20" s="38" t="n"/>
-      <c r="H20" s="38" t="n"/>
+      <c r="B19" s="38" t="n"/>
+      <c r="C19" s="38" t="n"/>
+      <c r="D19" s="38" t="n"/>
+      <c r="E19" s="38" t="n"/>
+      <c r="F19" s="38" t="n"/>
+      <c r="G19" s="38" t="n"/>
+      <c r="H19" s="38" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="39" t="inlineStr"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="39" t="inlineStr"/>
@@ -1590,58 +1544,48 @@
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="39" t="inlineStr"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="40" t="inlineStr">
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>“Düzenli çalışma, küçük adımların büyük sonuçlara dönüşmesidir.”</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="41" t="inlineStr">
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="14" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
         <is>
           <t>TED Okulları  |  Rehberlik Servisi  |  Hazırlayan: Merve Çelik</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A26:H26"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
@@ -1654,7 +1598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1677,7 +1621,7 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="44" t="inlineStr">
         <is>
-          <t>Program 17:30 okul çıkışından 22:00 uyku saatine kadar sabit bir çerçeve üzerine kuruludur: Günlük Ödev + Günlük Tekrar toplam 1.5 saat, Ek Çalışma (3 blok) toplam 2 saat. İhtiyaca göre 2-3 saat aralığında uzatılabilir; bunun için Ek Çalışma bloklarının süresini ve Mola/Yemek sürelerini kısaltıp uzatarak yeniden dengeleyebilirsiniz.</t>
+          <t>17:30 okul çıkışından 22:00 uyku saatine kadar 270 dakikalık sabit bir pencere kullanılır: 1 saat dinlenme + 1.5 saat günlük ödev/tekrar + 1.5 saat ek çalışma + kısa molalar + yemek + yatış hazırlığı tam olarak bu süreye oturacak şekilde ayarlanmıştır.</t>
         </is>
       </c>
     </row>
@@ -1691,75 +1635,89 @@
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="44" t="inlineStr">
         <is>
-          <t>Her hücredeki saat aralığını (örn. 18:35–19:20) doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
+          <t>Her hücredeki saat aralığını (örn. 19:20–20:05) doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="43" t="inlineStr">
         <is>
-          <t>• Ek Çalışma İçeriği</t>
+          <t>• Süreleri Yeniden Dengeleme</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="44" t="inlineStr">
         <is>
-          <t>"Ek Çalışma 1/2/3" satırlarındaki hücrelere dersin adını ve çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
+          <t>Bir bloğun süresini uzatmak isterseniz (örn. Ek Çalışmayı 1.5 saatten 2 saate çıkarmak), başka bir bloktan (mola, yemek veya dinlenme) o kadar dakika kısarak toplamı 270 dakikada sabit tutmanız gerekir; aksi halde 22:00 uyku hedefi kayar.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>• Uyku Saati</t>
+          <t>• Ek Çalışma İçeriği</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="44" t="inlineStr">
         <is>
-          <t>Program 22:00'de uyku hedefiyle tasarlanmıştır. Yatış saatini değiştirmek isterseniz son satırdaki "Yatış Hazırlığı" bloğunun saatini güncelleyip diğer blokları buna göre kaydırın.</t>
+          <t>"Ek Çalışma 1/2" satırlarındaki hücrelere dersin adını ve çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="43" t="inlineStr">
         <is>
-          <t>• Hafta İçi / Hafta Sonu</t>
+          <t>• Uyku Saati</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="44" t="inlineStr">
         <is>
-          <t>Program şu an tüm hafta için aynı saat şablonunu kullanır (tutarlı uyku düzeni için). Hafta sonu daha esnek olmasını isterseniz Cumartesi/Pazar sütunlarındaki saatleri ayrı ayrı değiştirebilirsiniz.</t>
+          <t>Program 22:00'de uyku hedefiyle tasarlanmıştır. Yatış saatini değiştirmek isterseniz son satırdaki "Yatış Hazırlığı" bloğunun saatini güncelleyip diğer blokları buna göre kaydırın.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="43" t="inlineStr">
         <is>
-          <t>• Renk Kodları</t>
+          <t>• Hafta İçi / Hafta Sonu</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="44" t="inlineStr">
         <is>
-          <t>Her blok türü farklı bir renkle gösterilir (bkz. sayfa üstündeki 'Renk Kodları' satırları).</t>
+          <t>Program şu an tüm hafta için aynı saat şablonunu kullanır (tutarlı uyku düzeni için). Hafta sonu daha esnek olmasını isterseniz Cumartesi/Pazar sütunlarındaki saatleri ayrı ayrı değiştirebilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="43" t="inlineStr">
         <is>
-          <t>• Logo Alanı</t>
+          <t>• Renk Kodları</t>
         </is>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="44" t="inlineStr">
+        <is>
+          <t>Her blok türü farklı bir renkle gösterilir (bkz. sayfa üstündeki 'Renk Kodları' satırları).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>• Logo Alanı</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="44" t="inlineStr">
         <is>
           <t>Sol üst köşedeki gri kutu TED okul logosu için ayrılmıştır. Logo görseli temin edildiğinde Ekle &gt; Resim ile bu alana yerleştirilebilir.</t>
         </is>

</xml_diff>

<commit_message>
Cumartesi-Pazar'ı gün boyu programa çevir, her güne kitap okuma ekle
Hafta sonu artık ayrı bir tabloda 09:00 uyanıştan 22:00 uykuya kadar
tam gün akışıyla planlanıyor: sabah 2 ek çalışma bloğu + ödev/proje,
uzun öğle+serbest zaman, akşamüstü tekrar, akşam yemeği+serbest zaman.
Hafta içi ve hafta sonu programlarının her ikisine de sabit bir
"Kitap Okuma" bloğu eklendi (hafta içi 15 dk, hafta sonu 30 dk).
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7UkXbn3U8T5AXkNxv5cKV
</commit_message>
<xml_diff>
--- a/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
+++ b/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Nasıl Düzenlenir" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Haftalik Program'!$A$1:$H$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="49">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,7 +45,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3B57"/>
-      <sz val="12"/>
+      <sz val="11.5"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -119,6 +119,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="006D1F35"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005C5041"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
@@ -126,7 +138,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11.5"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -138,6 +156,93 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="0037474F"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A237E"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00455A64"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00BF360C"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000D47A1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B5E20"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00827717"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="004A148C"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0000695C"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="006D1F35"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00311B92"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0037474F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00BF360C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00455A64"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="004A148C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B5E20"/>
       <sz val="10"/>
     </font>
     <font>
@@ -148,38 +253,19 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00455A64"/>
+      <color rgb="005C5041"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00BF360C"/>
+      <b val="1"/>
+      <color rgb="0000695C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000D47A1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001B5E20"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00827717"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="004A148C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="0000695C"/>
+      <b val="1"/>
+      <color rgb="006D1F35"/>
       <sz val="10"/>
     </font>
     <font>
@@ -220,7 +306,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -319,6 +405,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F6E2E7"/>
+        <bgColor rgb="00F6E2E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEAE3"/>
+        <bgColor rgb="00EFEAE3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003C5E82"/>
+        <bgColor rgb="003C5E82"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3B57"/>
         <bgColor rgb="001F3B57"/>
       </patternFill>
@@ -356,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -410,65 +514,122 @@
     <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="45" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -837,17 +998,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="15.5" customWidth="1" min="2" max="2"/>
+    <col width="15.5" customWidth="1" min="3" max="3"/>
+    <col width="15.5" customWidth="1" min="4" max="4"/>
+    <col width="15.5" customWidth="1" min="5" max="5"/>
+    <col width="15.5" customWidth="1" min="6" max="6"/>
+    <col width="15.5" customWidth="1" min="7" max="7"/>
+    <col width="15.5" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -875,7 +1036,7 @@
       <c r="A2" s="4" t="n"/>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Rehber Öğretmen: Merve Çelik   |   17:30 Okul Çıkışı → 1 sa Dinlenme → 22:00 Uyku</t>
+          <t>Rehber Öğretmen: Merve Çelik   |   Hafta İçi: 17:30 Çıkış → 22:00 Uyku   |   Hafta Sonu: Gün Boyu Program</t>
         </is>
       </c>
       <c r="C2" s="6" t="n"/>
@@ -963,632 +1124,900 @@
           <t>Yatış Hazırlığı</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr"/>
-      <c r="F5" s="21" t="inlineStr"/>
-      <c r="G5" s="21" t="inlineStr"/>
-      <c r="H5" s="21" t="inlineStr"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Serbest Zaman</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr"/>
+      <c r="H5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>HAFTA İÇİ PROGRAMI  (Pazartesi – Cuma)   ·   17:30 Okul Çıkışı → 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="25" t="n"/>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="25" t="n"/>
+      <c r="G6" s="25" t="n"/>
+      <c r="H6" s="25" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Zaman Bloğu</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>Pazartesi</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Salı</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Çarşamba</t>
         </is>
       </c>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>Perşembe</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>Cuma</t>
         </is>
       </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>Cumartesi</t>
-        </is>
-      </c>
-      <c r="H6" s="23" t="inlineStr">
-        <is>
-          <t>Pazar</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="G7" s="28" t="inlineStr"/>
+      <c r="H7" s="28" t="inlineStr"/>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Giriş / Dinlenme</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>17:30–18:30
 Eve Varış /
 Dinlenme (1 sa)</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>17:30–18:30
 Eve Varış /
 Dinlenme (1 sa)</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>17:30–18:30
 Eve Varış /
 Dinlenme (1 sa)</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>17:30–18:30
 Eve Varış /
 Dinlenme (1 sa)</t>
         </is>
       </c>
-      <c r="F7" s="25" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>17:30–18:30
 Eve Varış /
 Dinlenme (1 sa)</t>
         </is>
       </c>
-      <c r="G7" s="25" t="inlineStr">
-        <is>
-          <t>17:30–18:30
-Eve Varış /
-Dinlenme (1 sa)</t>
-        </is>
-      </c>
-      <c r="H7" s="25" t="inlineStr">
-        <is>
-          <t>17:30–18:30
-Eve Varış /
-Dinlenme (1 sa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="G8" s="28" t="inlineStr"/>
+      <c r="H8" s="28" t="inlineStr"/>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Günlük Ödev</t>
         </is>
       </c>
-      <c r="B8" s="26" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
 Günlük Ödevler</t>
         </is>
       </c>
-      <c r="G8" s="26" t="inlineStr">
-        <is>
-          <t>18:30–19:15
-Günlük Ödevler</t>
-        </is>
-      </c>
-      <c r="H8" s="26" t="inlineStr">
-        <is>
-          <t>18:30–19:15
-Günlük Ödevler</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="G9" s="28" t="inlineStr"/>
+      <c r="H9" s="28" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Mola</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="C9" s="27" t="inlineStr">
+Mola</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="D9" s="27" t="inlineStr">
+Mola</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="E9" s="27" t="inlineStr">
+Mola</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="inlineStr">
+Mola</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
         <is>
           <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="G9" s="27" t="inlineStr">
-        <is>
-          <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="H9" s="27" t="inlineStr">
-        <is>
-          <t>19:15–19:20
-Kısa Mola</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
+Mola</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr"/>
+      <c r="H10" s="28" t="inlineStr"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Ek Çalışma 1</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
-        <is>
-          <t>19:20–20:05
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>19:20–20:00
 Matematik
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>19:20–20:05
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>19:20–20:00
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>19:20–20:05
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>19:20–20:00
 Matematik
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="E10" s="29" t="inlineStr">
-        <is>
-          <t>19:20–20:05
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>19:20–20:00
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="F10" s="30" t="inlineStr">
-        <is>
-          <t>19:20–20:05
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>19:20–20:00
 Fen Bilimleri
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G10" s="28" t="inlineStr">
-        <is>
-          <t>19:20–20:05
-Matematik
-Yanlış Analizi</t>
-        </is>
-      </c>
-      <c r="H10" s="28" t="inlineStr">
-        <is>
-          <t>19:20–20:05
-Matematik
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="G11" s="28" t="inlineStr"/>
+      <c r="H11" s="28" t="inlineStr"/>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Yemek</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>20:00–20:15
 Yemek</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
+      <c r="C12" s="36" t="inlineStr">
+        <is>
+          <t>20:00–20:15
 Yemek</t>
         </is>
       </c>
-      <c r="D11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>20:00–20:15
 Yemek</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>20:00–20:15
 Yemek</t>
         </is>
       </c>
-      <c r="F11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
+      <c r="F12" s="36" t="inlineStr">
+        <is>
+          <t>20:00–20:15
 Yemek</t>
         </is>
       </c>
-      <c r="G11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
-Yemek</t>
-        </is>
-      </c>
-      <c r="H11" s="31" t="inlineStr">
-        <is>
-          <t>20:05–20:20
-Yemek</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="G12" s="28" t="inlineStr"/>
+      <c r="H12" s="28" t="inlineStr"/>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Ek Çalışma 2</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>20:20–21:05
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>20:15–20:50
 Türkçe
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="C12" s="28" t="inlineStr">
-        <is>
-          <t>20:20–21:05
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>20:15–20:50
 Matematik
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
-        <is>
-          <t>20:20–21:05
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>20:15–20:50
 Fen Bilimleri
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
-        <is>
-          <t>20:20–21:05
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>20:15–20:50
 Sosyal Bilgiler
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>20:20–21:05
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>20:15–20:50
 Türkçe
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G12" s="32" t="inlineStr">
-        <is>
-          <t>20:20–21:05
-Sosyal Bilgiler
-Soru Çözümü</t>
-        </is>
-      </c>
-      <c r="H12" s="30" t="inlineStr">
-        <is>
-          <t>20:20–21:05
-Fen Bil. &amp; Sosyal Bil.
-Genel Tekrar</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="G13" s="28" t="inlineStr"/>
+      <c r="H13" s="28" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Mola</t>
         </is>
       </c>
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="C13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="D13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="E13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="G13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-      <c r="H13" s="27" t="inlineStr">
-        <is>
-          <t>21:05–21:10
-Kısa Mola</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>20:50–20:55
+Mola</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>20:50–20:55
+Mola</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>20:50–20:55
+Mola</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>20:50–20:55
+Mola</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>20:50–20:55
+Mola</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr"/>
+      <c r="H14" s="28" t="inlineStr"/>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Günlük Tekrar</t>
         </is>
       </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>20:55–21:40
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>20:55–21:40
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>20:55–21:40
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>20:55–21:40
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="F14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>20:55–21:40
 Günlük Tekrar
 (Bugünkü konuların özeti)</t>
         </is>
       </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-      <c r="H14" s="33" t="inlineStr">
-        <is>
-          <t>21:10–21:55
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="G15" s="28" t="inlineStr"/>
+      <c r="H15" s="28" t="inlineStr"/>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>21:40–21:55
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>21:40–21:55
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="inlineStr">
+        <is>
+          <t>21:40–21:55
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>21:40–21:55
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>21:40–21:55
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr"/>
+      <c r="H16" s="28" t="inlineStr"/>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Yatış Hazırlığı</t>
         </is>
       </c>
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C17" s="40" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="D15" s="34" t="inlineStr">
+      <c r="D17" s="40" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="E15" s="34" t="inlineStr">
+      <c r="E17" s="40" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="F15" s="34" t="inlineStr">
+      <c r="F17" s="40" t="inlineStr">
         <is>
           <t>21:55–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="G15" s="34" t="inlineStr">
-        <is>
-          <t>21:55–22:00
+      <c r="G17" s="28" t="inlineStr"/>
+      <c r="H17" s="28" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>HAFTA SONU PROGRAMI  (Cumartesi – Pazar)   ·   Gün Boyu  ·  09:00 Uyanış → 22:00 Uyku</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Zaman Bloğu</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>Cumartesi</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="42" t="n"/>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>Pazar</t>
+        </is>
+      </c>
+      <c r="F20" s="42" t="n"/>
+      <c r="G20" s="42" t="n"/>
+      <c r="H20" s="28" t="inlineStr"/>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>Uyanış / Kahvaltı</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>09:00–09:30
+Uyanış / Kahvaltı</t>
+        </is>
+      </c>
+      <c r="C21" s="44" t="n"/>
+      <c r="D21" s="44" t="n"/>
+      <c r="E21" s="43" t="inlineStr">
+        <is>
+          <t>09:00–09:30
+Uyanış / Kahvaltı</t>
+        </is>
+      </c>
+      <c r="F21" s="44" t="n"/>
+      <c r="G21" s="44" t="n"/>
+      <c r="H21" s="28" t="inlineStr"/>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 1</t>
+        </is>
+      </c>
+      <c r="B22" s="45" t="inlineStr">
+        <is>
+          <t>09:30–10:15
+Matematik
+Yanlış Analizi</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="n"/>
+      <c r="D22" s="46" t="n"/>
+      <c r="E22" s="45" t="inlineStr">
+        <is>
+          <t>09:30–10:15
+Matematik
+Genel Tekrar</t>
+        </is>
+      </c>
+      <c r="F22" s="46" t="n"/>
+      <c r="G22" s="46" t="n"/>
+      <c r="H22" s="28" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B23" s="47" t="inlineStr">
+        <is>
+          <t>10:15–10:25
+Mola</t>
+        </is>
+      </c>
+      <c r="C23" s="48" t="n"/>
+      <c r="D23" s="48" t="n"/>
+      <c r="E23" s="47" t="inlineStr">
+        <is>
+          <t>10:15–10:25
+Mola</t>
+        </is>
+      </c>
+      <c r="F23" s="48" t="n"/>
+      <c r="G23" s="48" t="n"/>
+      <c r="H23" s="28" t="inlineStr"/>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 2</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>10:25–11:10
+Sosyal Bilgiler
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="C24" s="50" t="n"/>
+      <c r="D24" s="50" t="n"/>
+      <c r="E24" s="51" t="inlineStr">
+        <is>
+          <t>10:25–11:10
+Fen Bil. &amp; Sosyal Bil.
+Genel Tekrar</t>
+        </is>
+      </c>
+      <c r="F24" s="52" t="n"/>
+      <c r="G24" s="52" t="n"/>
+      <c r="H24" s="28" t="inlineStr"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Ödev / Proje</t>
+        </is>
+      </c>
+      <c r="B25" s="53" t="inlineStr">
+        <is>
+          <t>11:10–12:00
+Günlük Ödev /
+Proje Çalışması</t>
+        </is>
+      </c>
+      <c r="C25" s="54" t="n"/>
+      <c r="D25" s="54" t="n"/>
+      <c r="E25" s="53" t="inlineStr">
+        <is>
+          <t>11:10–12:00
+Haftaya Hazırlık
+(Çanta, Kıyafet vb.)</t>
+        </is>
+      </c>
+      <c r="F25" s="54" t="n"/>
+      <c r="G25" s="54" t="n"/>
+      <c r="H25" s="28" t="inlineStr"/>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Öğle + Serbest Zaman</t>
+        </is>
+      </c>
+      <c r="B26" s="55" t="inlineStr">
+        <is>
+          <t>12:00–16:00
+Öğle Yemeği +
+Serbest Zaman
+(Aile / Hobi / Spor)</t>
+        </is>
+      </c>
+      <c r="C26" s="56" t="n"/>
+      <c r="D26" s="56" t="n"/>
+      <c r="E26" s="55" t="inlineStr">
+        <is>
+          <t>12:00–16:00
+Öğle Yemeği +
+Serbest Zaman
+(Aile / Hobi / Spor)</t>
+        </is>
+      </c>
+      <c r="F26" s="56" t="n"/>
+      <c r="G26" s="56" t="n"/>
+      <c r="H26" s="28" t="inlineStr"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Günlük Tekrar</t>
+        </is>
+      </c>
+      <c r="B27" s="57" t="inlineStr">
+        <is>
+          <t>16:00–16:45
+Günlük Tekrar</t>
+        </is>
+      </c>
+      <c r="C27" s="58" t="n"/>
+      <c r="D27" s="58" t="n"/>
+      <c r="E27" s="57" t="inlineStr">
+        <is>
+          <t>16:00–16:45
+Haftalık Genel
+Değerlendirme</t>
+        </is>
+      </c>
+      <c r="F27" s="58" t="n"/>
+      <c r="G27" s="58" t="n"/>
+      <c r="H27" s="28" t="inlineStr"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="B28" s="59" t="inlineStr">
+        <is>
+          <t>16:45–17:15
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="C28" s="60" t="n"/>
+      <c r="D28" s="60" t="n"/>
+      <c r="E28" s="59" t="inlineStr">
+        <is>
+          <t>16:45–17:15
+Kitap Okuma</t>
+        </is>
+      </c>
+      <c r="F28" s="60" t="n"/>
+      <c r="G28" s="60" t="n"/>
+      <c r="H28" s="28" t="inlineStr"/>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>Akşam + Serbest Zaman</t>
+        </is>
+      </c>
+      <c r="B29" s="55" t="inlineStr">
+        <is>
+          <t>17:15–21:30
+Akşam Yemeği +
+Serbest Zaman / Aile</t>
+        </is>
+      </c>
+      <c r="C29" s="56" t="n"/>
+      <c r="D29" s="56" t="n"/>
+      <c r="E29" s="55" t="inlineStr">
+        <is>
+          <t>17:15–21:30
+Akşam Yemeği +
+Serbest Zaman / Aile</t>
+        </is>
+      </c>
+      <c r="F29" s="56" t="n"/>
+      <c r="G29" s="56" t="n"/>
+      <c r="H29" s="28" t="inlineStr"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Yatış Hazırlığı</t>
+        </is>
+      </c>
+      <c r="B30" s="61" t="inlineStr">
+        <is>
+          <t>21:30–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>21:55–22:00
+      <c r="C30" s="62" t="n"/>
+      <c r="D30" s="62" t="n"/>
+      <c r="E30" s="61" t="inlineStr">
+        <is>
+          <t>21:30–22:00
 Yatış Hazırlığı
 → 22:00 Uyku</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="35" t="inlineStr">
-        <is>
-          <t>Haftalık Ek Çalışma Dağılımı  —  Matematik: 5  |  Türkçe: 4  |  Fen Bilimleri: 3  |  Sosyal Bilgiler: 2   (Dinlenme: 1 saat, Günlük Ödev + Günlük Tekrar: 1.5 saat, Ek Çalışma: 1.5 saat/gün, Uyku: 22:00)</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="n"/>
-      <c r="C17" s="36" t="n"/>
-      <c r="D17" s="36" t="n"/>
-      <c r="E17" s="36" t="n"/>
-      <c r="F17" s="36" t="n"/>
-      <c r="G17" s="36" t="n"/>
-      <c r="H17" s="36" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="F30" s="62" t="n"/>
+      <c r="G30" s="62" t="n"/>
+      <c r="H30" s="28" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="63" t="inlineStr">
+        <is>
+          <t>Haftalık Ek Çalışma Dağılımı  —  Matematik: 5  |  Türkçe: 4  |  Fen Bilimleri: 3  |  Sosyal Bilgiler: 2   ·   Kitap Okuma: 7 gün / 7 gün   ·   Uyku: Her gün 22:00</t>
+        </is>
+      </c>
+      <c r="B32" s="64" t="n"/>
+      <c r="C32" s="64" t="n"/>
+      <c r="D32" s="64" t="n"/>
+      <c r="E32" s="64" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="64" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="65" t="inlineStr">
         <is>
           <t>NOTLAR</t>
         </is>
       </c>
-      <c r="B19" s="38" t="n"/>
-      <c r="C19" s="38" t="n"/>
-      <c r="D19" s="38" t="n"/>
-      <c r="E19" s="38" t="n"/>
-      <c r="F19" s="38" t="n"/>
-      <c r="G19" s="38" t="n"/>
-      <c r="H19" s="38" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="39" t="inlineStr"/>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
-      <c r="H20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="39" t="inlineStr"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="39" t="inlineStr"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="8" t="n"/>
-    </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="40" t="inlineStr">
+      <c r="B34" s="42" t="n"/>
+      <c r="C34" s="42" t="n"/>
+      <c r="D34" s="42" t="n"/>
+      <c r="E34" s="42" t="n"/>
+      <c r="F34" s="42" t="n"/>
+      <c r="G34" s="42" t="n"/>
+      <c r="H34" s="42" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="66" t="inlineStr"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="66" t="inlineStr"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="66" t="inlineStr"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="67" t="inlineStr">
         <is>
           <t>“Düzenli çalışma, küçük adımların büyük sonuçlara dönüşmesidir.”</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-    </row>
-    <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+    </row>
+    <row r="40" ht="14" customHeight="1">
+      <c r="A40" s="68" t="inlineStr">
         <is>
           <t>TED Okulları  |  Rehberlik Servisi  |  Hazırlayan: Merve Çelik</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="36">
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B20:D20"/>
     <mergeCell ref="A1:A3"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A35:H35"/>
     <mergeCell ref="B1:H1"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+  <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1605,119 +2034,119 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="69" t="inlineStr">
         <is>
           <t>Programı Nasıl Düzenlersiniz?</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="43" t="inlineStr">
-        <is>
-          <t>• Zaman Yapısı</t>
+      <c r="A3" s="70" t="inlineStr">
+        <is>
+          <t>• İki Ayrı Tablo</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
-        <is>
-          <t>17:30 okul çıkışından 22:00 uyku saatine kadar 270 dakikalık sabit bir pencere kullanılır: 1 saat dinlenme + 1.5 saat günlük ödev/tekrar + 1.5 saat ek çalışma + kısa molalar + yemek + yatış hazırlığı tam olarak bu süreye oturacak şekilde ayarlanmıştır.</t>
+      <c r="A4" s="71" t="inlineStr">
+        <is>
+          <t>Hafta içi (Pazartesi–Cuma) 17:30–22:00 arası okul sonrası akışını, hafta sonu (Cumartesi–Pazar) ise 09:00–22:00 arası gün boyu akışını gösterir. İki tablo farklı saat yapıları kullandığı için ayrı gösterilmiştir.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>• Kitap Okuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>Her gün (hafta içi 15 dk, hafta sonu 30 dk) sabit bir 'Kitap Okuma' bloğu bulunur. Süresini veya saatini değiştirmek isterseniz ilgili hücreyi ve komşu bloğun süresini birlikte güncelleyin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="70" t="inlineStr">
         <is>
           <t>• Ders Saatleri</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
-        <is>
-          <t>Her hücredeki saat aralığını (örn. 19:20–20:05) doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="43" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>Her hücredeki saat aralığını doğrudan tıklayıp yazarak değiştirebilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
         <is>
           <t>• Süreleri Yeniden Dengeleme</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="44" t="inlineStr">
-        <is>
-          <t>Bir bloğun süresini uzatmak isterseniz (örn. Ek Çalışmayı 1.5 saatten 2 saate çıkarmak), başka bir bloktan (mola, yemek veya dinlenme) o kadar dakika kısarak toplamı 270 dakikada sabit tutmanız gerekir; aksi halde 22:00 uyku hedefi kayar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Bir bloğun süresini uzatmak isterseniz başka bir bloktan o kadar dakika kısarak toplamı hafta içi için 270 dakikada (17:30-22:00), hafta sonu için 780 dakikada (09:00-22:00) sabit tutmanız gerekir; aksi halde 22:00 uyku hedefi kayar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
+          <t>• Hafta Sonu Serbest Zaman</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="71" t="inlineStr">
+        <is>
+          <t>Cumartesi/Pazar'daki geniş 'Öğle + Serbest Zaman' ve 'Akşam + Serbest Zaman' blokları aile, hobi, spor gibi etkinlikler için ayrılmıştır; içeriğini dilediğiniz gibi değiştirebilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="70" t="inlineStr">
         <is>
           <t>• Ek Çalışma İçeriği</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="44" t="inlineStr">
-        <is>
-          <t>"Ek Çalışma 1/2" satırlarındaki hücrelere dersin adını ve çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="43" t="inlineStr">
-        <is>
-          <t>• Uyku Saati</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="44" t="inlineStr">
-        <is>
-          <t>Program 22:00'de uyku hedefiyle tasarlanmıştır. Yatış saatini değiştirmek isterseniz son satırdaki "Yatış Hazırlığı" bloğunun saatini güncelleyip diğer blokları buna göre kaydırın.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
-        <is>
-          <t>• Hafta İçi / Hafta Sonu</t>
-        </is>
-      </c>
-    </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
-        <is>
-          <t>Program şu an tüm hafta için aynı saat şablonunu kullanır (tutarlı uyku düzeni için). Hafta sonu daha esnek olmasını isterseniz Cumartesi/Pazar sütunlarındaki saatleri ayrı ayrı değiştirebilirsiniz.</t>
+      <c r="A19" s="71" t="inlineStr">
+        <is>
+          <t>"Ek Çalışma 1/2" hücrelerine dersin adını ve çalışma türünü (konu tekrarı, soru çözümü, test, yanlış analizi vb.) yazabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="43" t="inlineStr">
+      <c r="A21" s="70" t="inlineStr">
         <is>
           <t>• Renk Kodları</t>
         </is>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="44" t="inlineStr">
+      <c r="A22" s="71" t="inlineStr">
         <is>
           <t>Her blok türü farklı bir renkle gösterilir (bkz. sayfa üstündeki 'Renk Kodları' satırları).</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="43" t="inlineStr">
+      <c r="A24" s="70" t="inlineStr">
         <is>
           <t>• Logo Alanı</t>
         </is>
       </c>
     </row>
     <row r="25" ht="34" customHeight="1">
-      <c r="A25" s="44" t="inlineStr">
+      <c r="A25" s="71" t="inlineStr">
         <is>
           <t>Sol üst köşedeki gri kutu TED okul logosu için ayrılmıştır. Logo görseli temin edildiğinde Ekle &gt; Resim ile bu alana yerleştirilebilir.</t>
         </is>

</xml_diff>

<commit_message>
Günlük akışı Tekrar → Ödev → Ek Çalışma → Kitap Okuma sırasına göre yeniden düzenle
Hem hafta içi hem hafta sonu tablosunda bloklar artık önce günlük
tekrar, sonra günlük ödev, ardından ek çalışma, en son kitap okuma
şeklinde ilerliyor. Giriş/dinlenme en başta, yatış hazırlığı en
sonda kalmaya devam ediyor; toplam süreler (270 dk hafta içi,
780 dk hafta sonu) değişmedi.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7UkXbn3U8T5AXkNxv5cKV
</commit_message>
<xml_diff>
--- a/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
+++ b/7_Sinif_Haftalik_Ders_Calisma_Programi.xlsx
@@ -160,6 +160,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="0000695C"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="001A237E"/>
       <sz val="9.5"/>
     </font>
@@ -197,11 +202,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000695C"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="006D1F35"/>
       <sz val="9.5"/>
@@ -226,13 +226,30 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0000695C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A237E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00455A64"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00BF360C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00455A64"/>
+      <color rgb="005C5041"/>
       <sz val="10"/>
     </font>
     <font>
@@ -243,23 +260,6 @@
     <font>
       <name val="Arial"/>
       <color rgb="001B5E20"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001A237E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="005C5041"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0000695C"/>
       <sz val="10"/>
     </font>
     <font>
@@ -538,28 +538,28 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -576,34 +576,34 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="38" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="40" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="42" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1232,286 +1232,286 @@
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Günlük Ödev</t>
+          <t>Günlük Tekrar</t>
         </is>
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
-Günlük Ödevler</t>
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
         </is>
       </c>
       <c r="C9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
-Günlük Ödevler</t>
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
         </is>
       </c>
       <c r="D9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
-Günlük Ödevler</t>
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
         </is>
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
-Günlük Ödevler</t>
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
         <is>
           <t>18:30–19:15
-Günlük Ödevler</t>
+Günlük Tekrar
+(Bugünkü konuların özeti)</t>
         </is>
       </c>
       <c r="G9" s="28" t="inlineStr"/>
       <c r="H9" s="28" t="inlineStr"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Mola</t>
+          <t>Günlük Ödev</t>
         </is>
       </c>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>19:15–19:20
-Mola</t>
+          <t>19:15–20:00
+Günlük Ödevler</t>
         </is>
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>19:15–19:20
-Mola</t>
+          <t>19:15–20:00
+Günlük Ödevler</t>
         </is>
       </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
-          <t>19:15–19:20
-Mola</t>
+          <t>19:15–20:00
+Günlük Ödevler</t>
         </is>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
-          <t>19:15–19:20
-Mola</t>
+          <t>19:15–20:00
+Günlük Ödevler</t>
         </is>
       </c>
       <c r="F10" s="32" t="inlineStr">
         <is>
-          <t>19:15–19:20
-Mola</t>
+          <t>19:15–20:00
+Günlük Ödevler</t>
         </is>
       </c>
       <c r="G10" s="28" t="inlineStr"/>
       <c r="H10" s="28" t="inlineStr"/>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="29" t="inlineStr">
         <is>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>20:00–20:05
+Mola</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>20:00–20:05
+Mola</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>20:00–20:05
+Mola</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>20:00–20:05
+Mola</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>20:00–20:05
+Mola</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="inlineStr"/>
+      <c r="H11" s="28" t="inlineStr"/>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
           <t>Ek Çalışma 1</t>
         </is>
       </c>
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="B12" s="34" t="inlineStr">
+        <is>
+          <t>20:05–20:45
 Matematik
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>20:05–20:45
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>20:05–20:45
 Matematik
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="E11" s="34" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>20:05–20:45
 Türkçe
 Konu Tekrarı</t>
         </is>
       </c>
-      <c r="F11" s="35" t="inlineStr">
-        <is>
-          <t>19:20–20:00
+      <c r="F12" s="36" t="inlineStr">
+        <is>
+          <t>20:05–20:45
 Fen Bilimleri
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G11" s="28" t="inlineStr"/>
-      <c r="H11" s="28" t="inlineStr"/>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
-        <is>
-          <t>Yemek</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="inlineStr">
-        <is>
-          <t>20:00–20:15
-Yemek</t>
-        </is>
-      </c>
-      <c r="C12" s="36" t="inlineStr">
-        <is>
-          <t>20:00–20:15
-Yemek</t>
-        </is>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>20:00–20:15
-Yemek</t>
-        </is>
-      </c>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>20:00–20:15
-Yemek</t>
-        </is>
-      </c>
-      <c r="F12" s="36" t="inlineStr">
-        <is>
-          <t>20:00–20:15
-Yemek</t>
-        </is>
-      </c>
       <c r="G12" s="28" t="inlineStr"/>
       <c r="H12" s="28" t="inlineStr"/>
     </row>
-    <row r="13" ht="52" customHeight="1">
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="29" t="inlineStr">
         <is>
+          <t>Yemek</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>20:45–21:00
+Yemek</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>20:45–21:00
+Yemek</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>20:45–21:00
+Yemek</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>20:45–21:00
+Yemek</t>
+        </is>
+      </c>
+      <c r="F13" s="37" t="inlineStr">
+        <is>
+          <t>20:45–21:00
+Yemek</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="inlineStr"/>
+      <c r="H13" s="28" t="inlineStr"/>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
           <t>Ek Çalışma 2</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
-        <is>
-          <t>20:15–20:50
+      <c r="B14" s="35" t="inlineStr">
+        <is>
+          <t>21:00–21:35
 Türkçe
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>20:15–20:50
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>21:00–21:35
 Matematik
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>20:15–20:50
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>21:00–21:35
 Fen Bilimleri
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="E13" s="37" t="inlineStr">
-        <is>
-          <t>20:15–20:50
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>21:00–21:35
 Sosyal Bilgiler
 Soru Çözümü</t>
         </is>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>20:15–20:50
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>21:00–21:35
 Türkçe
 Test Çözümü</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr"/>
-      <c r="H13" s="28" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Mola</t>
-        </is>
-      </c>
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t>20:50–20:55
-Mola</t>
-        </is>
-      </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>20:50–20:55
-Mola</t>
-        </is>
-      </c>
-      <c r="D14" s="32" t="inlineStr">
-        <is>
-          <t>20:50–20:55
-Mola</t>
-        </is>
-      </c>
-      <c r="E14" s="32" t="inlineStr">
-        <is>
-          <t>20:50–20:55
-Mola</t>
-        </is>
-      </c>
-      <c r="F14" s="32" t="inlineStr">
-        <is>
-          <t>20:50–20:55
-Mola</t>
-        </is>
-      </c>
       <c r="G14" s="28" t="inlineStr"/>
       <c r="H14" s="28" t="inlineStr"/>
     </row>
-    <row r="15" ht="44" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>Günlük Tekrar</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
-        <is>
-          <t>20:55–21:40
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-      <c r="C15" s="38" t="inlineStr">
-        <is>
-          <t>20:55–21:40
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-      <c r="D15" s="38" t="inlineStr">
-        <is>
-          <t>20:55–21:40
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>20:55–21:40
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
-        </is>
-      </c>
-      <c r="F15" s="38" t="inlineStr">
-        <is>
-          <t>20:55–21:40
-Günlük Tekrar
-(Bugünkü konuların özeti)</t>
+          <t>Mola</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>21:35–21:40
+Mola</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>21:35–21:40
+Mola</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>21:35–21:40
+Mola</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>21:35–21:40
+Mola</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>21:35–21:40
+Mola</t>
         </is>
       </c>
       <c r="G15" s="28" t="inlineStr"/>
@@ -1660,17 +1660,16 @@
       <c r="G21" s="44" t="n"/>
       <c r="H21" s="28" t="inlineStr"/>
     </row>
-    <row r="22" ht="50" customHeight="1">
+    <row r="22" ht="40" customHeight="1">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>Ek Çalışma 1</t>
+          <t>Günlük Tekrar</t>
         </is>
       </c>
       <c r="B22" s="45" t="inlineStr">
         <is>
           <t>09:30–10:15
-Matematik
-Yanlış Analizi</t>
+Günlük Tekrar</t>
         </is>
       </c>
       <c r="C22" s="46" t="n"/>
@@ -1678,88 +1677,88 @@
       <c r="E22" s="45" t="inlineStr">
         <is>
           <t>09:30–10:15
-Matematik
-Genel Tekrar</t>
+Haftalık Genel
+Değerlendirme</t>
         </is>
       </c>
       <c r="F22" s="46" t="n"/>
       <c r="G22" s="46" t="n"/>
       <c r="H22" s="28" t="inlineStr"/>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="40" customHeight="1">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t>Mola</t>
+          <t>Ödev / Proje</t>
         </is>
       </c>
       <c r="B23" s="47" t="inlineStr">
         <is>
-          <t>10:15–10:25
-Mola</t>
+          <t>10:15–11:00
+Günlük Ödev /
+Proje Çalışması</t>
         </is>
       </c>
       <c r="C23" s="48" t="n"/>
       <c r="D23" s="48" t="n"/>
       <c r="E23" s="47" t="inlineStr">
         <is>
-          <t>10:15–10:25
-Mola</t>
+          <t>10:15–11:00
+Haftaya Hazırlık
+(Çanta, Kıyafet vb.)</t>
         </is>
       </c>
       <c r="F23" s="48" t="n"/>
       <c r="G23" s="48" t="n"/>
       <c r="H23" s="28" t="inlineStr"/>
     </row>
-    <row r="24" ht="50" customHeight="1">
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>Ek Çalışma 2</t>
+          <t>Mola</t>
         </is>
       </c>
       <c r="B24" s="49" t="inlineStr">
         <is>
-          <t>10:25–11:10
-Sosyal Bilgiler
-Soru Çözümü</t>
+          <t>11:00–11:10
+Mola</t>
         </is>
       </c>
       <c r="C24" s="50" t="n"/>
       <c r="D24" s="50" t="n"/>
-      <c r="E24" s="51" t="inlineStr">
-        <is>
-          <t>10:25–11:10
-Fen Bil. &amp; Sosyal Bil.
+      <c r="E24" s="49" t="inlineStr">
+        <is>
+          <t>11:00–11:10
+Mola</t>
+        </is>
+      </c>
+      <c r="F24" s="50" t="n"/>
+      <c r="G24" s="50" t="n"/>
+      <c r="H24" s="28" t="inlineStr"/>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Ek Çalışma 1</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>11:10–11:55
+Matematik
+Yanlış Analizi</t>
+        </is>
+      </c>
+      <c r="C25" s="52" t="n"/>
+      <c r="D25" s="52" t="n"/>
+      <c r="E25" s="51" t="inlineStr">
+        <is>
+          <t>11:10–11:55
+Matematik
 Genel Tekrar</t>
         </is>
       </c>
-      <c r="F24" s="52" t="n"/>
-      <c r="G24" s="52" t="n"/>
-      <c r="H24" s="28" t="inlineStr"/>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="29" t="inlineStr">
-        <is>
-          <t>Ödev / Proje</t>
-        </is>
-      </c>
-      <c r="B25" s="53" t="inlineStr">
-        <is>
-          <t>11:10–12:00
-Günlük Ödev /
-Proje Çalışması</t>
-        </is>
-      </c>
-      <c r="C25" s="54" t="n"/>
-      <c r="D25" s="54" t="n"/>
-      <c r="E25" s="53" t="inlineStr">
-        <is>
-          <t>11:10–12:00
-Haftaya Hazırlık
-(Çanta, Kıyafet vb.)</t>
-        </is>
-      </c>
-      <c r="F25" s="54" t="n"/>
-      <c r="G25" s="54" t="n"/>
+      <c r="F25" s="52" t="n"/>
+      <c r="G25" s="52" t="n"/>
       <c r="H25" s="28" t="inlineStr"/>
     </row>
     <row r="26" ht="44" customHeight="1">
@@ -1768,47 +1767,48 @@
           <t>Öğle + Serbest Zaman</t>
         </is>
       </c>
-      <c r="B26" s="55" t="inlineStr">
-        <is>
-          <t>12:00–16:00
+      <c r="B26" s="53" t="inlineStr">
+        <is>
+          <t>11:55–15:55
 Öğle Yemeği +
 Serbest Zaman
 (Aile / Hobi / Spor)</t>
         </is>
       </c>
-      <c r="C26" s="56" t="n"/>
-      <c r="D26" s="56" t="n"/>
-      <c r="E26" s="55" t="inlineStr">
-        <is>
-          <t>12:00–16:00
+      <c r="C26" s="54" t="n"/>
+      <c r="D26" s="54" t="n"/>
+      <c r="E26" s="53" t="inlineStr">
+        <is>
+          <t>11:55–15:55
 Öğle Yemeği +
 Serbest Zaman
 (Aile / Hobi / Spor)</t>
         </is>
       </c>
-      <c r="F26" s="56" t="n"/>
-      <c r="G26" s="56" t="n"/>
+      <c r="F26" s="54" t="n"/>
+      <c r="G26" s="54" t="n"/>
       <c r="H26" s="28" t="inlineStr"/>
     </row>
-    <row r="27" ht="40" customHeight="1">
+    <row r="27" ht="50" customHeight="1">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>Günlük Tekrar</t>
-        </is>
-      </c>
-      <c r="B27" s="57" t="inlineStr">
-        <is>
-          <t>16:00–16:45
-Günlük Tekrar</t>
-        </is>
-      </c>
-      <c r="C27" s="58" t="n"/>
-      <c r="D27" s="58" t="n"/>
+          <t>Ek Çalışma 2</t>
+        </is>
+      </c>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t>15:55–16:40
+Sosyal Bilgiler
+Soru Çözümü</t>
+        </is>
+      </c>
+      <c r="C27" s="56" t="n"/>
+      <c r="D27" s="56" t="n"/>
       <c r="E27" s="57" t="inlineStr">
         <is>
-          <t>16:00–16:45
-Haftalık Genel
-Değerlendirme</t>
+          <t>15:55–16:40
+Fen Bil. &amp; Sosyal Bil.
+Genel Tekrar</t>
         </is>
       </c>
       <c r="F27" s="58" t="n"/>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B28" s="59" t="inlineStr">
         <is>
-          <t>16:45–17:15
+          <t>16:40–17:10
 Kitap Okuma</t>
         </is>
       </c>
@@ -1831,7 +1831,7 @@
       <c r="D28" s="60" t="n"/>
       <c r="E28" s="59" t="inlineStr">
         <is>
-          <t>16:45–17:15
+          <t>16:40–17:10
 Kitap Okuma</t>
         </is>
       </c>
@@ -1845,24 +1845,24 @@
           <t>Akşam + Serbest Zaman</t>
         </is>
       </c>
-      <c r="B29" s="55" t="inlineStr">
-        <is>
-          <t>17:15–21:30
+      <c r="B29" s="53" t="inlineStr">
+        <is>
+          <t>17:10–21:30
 Akşam Yemeği +
 Serbest Zaman / Aile</t>
         </is>
       </c>
-      <c r="C29" s="56" t="n"/>
-      <c r="D29" s="56" t="n"/>
-      <c r="E29" s="55" t="inlineStr">
-        <is>
-          <t>17:15–21:30
+      <c r="C29" s="54" t="n"/>
+      <c r="D29" s="54" t="n"/>
+      <c r="E29" s="53" t="inlineStr">
+        <is>
+          <t>17:10–21:30
 Akşam Yemeği +
 Serbest Zaman / Aile</t>
         </is>
       </c>
-      <c r="F29" s="56" t="n"/>
-      <c r="G29" s="56" t="n"/>
+      <c r="F29" s="54" t="n"/>
+      <c r="G29" s="54" t="n"/>
       <c r="H29" s="28" t="inlineStr"/>
     </row>
     <row r="30" ht="40" customHeight="1">

</xml_diff>